<commit_message>
Plantilla Excel: 12 meses y detalle semanal/diario del mes
</commit_message>
<xml_diff>
--- a/assets/plantilla-importacion-indicadores.xlsx
+++ b/assets/plantilla-importacion-indicadores.xlsx
@@ -430,7 +430,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2. Esta plantilla se genera con el mes de referencia: año 2026, mes 4 (2026-04).</v>
+        <v>2. Esta plantilla se genera con el mes de referencia: año 2026, mes 5 (2026-05).</v>
       </c>
     </row>
     <row r="6">
@@ -445,7 +445,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>4. En hojas *_detalle, tipo = semana (número de semana ISO) o dia (día del mes 1-30).</v>
+        <v>4. En hojas *_detalle, tipo = semana (número de semana ISO) o dia (día del mes 1-31).</v>
       </c>
     </row>
     <row r="9">
@@ -480,7 +480,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>carros_detalle — Semanas ISO que caen en 2026-04 + un día por fila (1-30)</v>
+        <v>carros_detalle — Semanas ISO que caen en 2026-05 + un día por fila (1-31)</v>
       </c>
     </row>
     <row r="16">
@@ -507,7 +507,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -528,13 +528,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B2" t="str">
         <v>semana</v>
       </c>
       <c r="C2">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -545,13 +545,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B3" t="str">
         <v>semana</v>
       </c>
       <c r="C3">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -562,13 +562,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B4" t="str">
         <v>semana</v>
       </c>
       <c r="C4">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -579,13 +579,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B5" t="str">
         <v>semana</v>
       </c>
       <c r="C5">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -596,13 +596,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B6" t="str">
         <v>semana</v>
       </c>
       <c r="C6">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -613,7 +613,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B7" t="str">
         <v>dia</v>
@@ -630,7 +630,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B8" t="str">
         <v>dia</v>
@@ -647,7 +647,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B9" t="str">
         <v>dia</v>
@@ -664,7 +664,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B10" t="str">
         <v>dia</v>
@@ -681,7 +681,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B11" t="str">
         <v>dia</v>
@@ -698,7 +698,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B12" t="str">
         <v>dia</v>
@@ -715,7 +715,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B13" t="str">
         <v>dia</v>
@@ -732,7 +732,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B14" t="str">
         <v>dia</v>
@@ -749,7 +749,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B15" t="str">
         <v>dia</v>
@@ -766,7 +766,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B16" t="str">
         <v>dia</v>
@@ -783,7 +783,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B17" t="str">
         <v>dia</v>
@@ -800,7 +800,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B18" t="str">
         <v>dia</v>
@@ -817,7 +817,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B19" t="str">
         <v>dia</v>
@@ -834,7 +834,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B20" t="str">
         <v>dia</v>
@@ -851,7 +851,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B21" t="str">
         <v>dia</v>
@@ -868,7 +868,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B22" t="str">
         <v>dia</v>
@@ -885,7 +885,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B23" t="str">
         <v>dia</v>
@@ -902,7 +902,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B24" t="str">
         <v>dia</v>
@@ -919,7 +919,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B25" t="str">
         <v>dia</v>
@@ -936,7 +936,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B26" t="str">
         <v>dia</v>
@@ -953,7 +953,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B27" t="str">
         <v>dia</v>
@@ -970,7 +970,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B28" t="str">
         <v>dia</v>
@@ -987,7 +987,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B29" t="str">
         <v>dia</v>
@@ -1004,7 +1004,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B30" t="str">
         <v>dia</v>
@@ -1021,7 +1021,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B31" t="str">
         <v>dia</v>
@@ -1038,7 +1038,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B32" t="str">
         <v>dia</v>
@@ -1055,7 +1055,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B33" t="str">
         <v>dia</v>
@@ -1072,7 +1072,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B34" t="str">
         <v>dia</v>
@@ -1089,7 +1089,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B35" t="str">
         <v>dia</v>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B36" t="str">
         <v>dia</v>
@@ -1121,9 +1121,26 @@
         <v/>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>2026-05</v>
+      </c>
+      <c r="B37" t="str">
+        <v>dia</v>
+      </c>
+      <c r="C37">
+        <v>31</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1399,7 +1416,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1429,13 +1446,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B2" t="str">
         <v>semana</v>
       </c>
       <c r="C2">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1455,13 +1472,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B3" t="str">
         <v>semana</v>
       </c>
       <c r="C3">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -1481,13 +1498,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B4" t="str">
         <v>semana</v>
       </c>
       <c r="C4">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -1507,13 +1524,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B5" t="str">
         <v>semana</v>
       </c>
       <c r="C5">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -1533,13 +1550,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B6" t="str">
         <v>semana</v>
       </c>
       <c r="C6">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -1559,7 +1576,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B7" t="str">
         <v>dia</v>
@@ -1585,7 +1602,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B8" t="str">
         <v>dia</v>
@@ -1611,7 +1628,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B9" t="str">
         <v>dia</v>
@@ -1637,7 +1654,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B10" t="str">
         <v>dia</v>
@@ -1663,7 +1680,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B11" t="str">
         <v>dia</v>
@@ -1689,7 +1706,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B12" t="str">
         <v>dia</v>
@@ -1715,7 +1732,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B13" t="str">
         <v>dia</v>
@@ -1741,7 +1758,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B14" t="str">
         <v>dia</v>
@@ -1767,7 +1784,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B15" t="str">
         <v>dia</v>
@@ -1793,7 +1810,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B16" t="str">
         <v>dia</v>
@@ -1819,7 +1836,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B17" t="str">
         <v>dia</v>
@@ -1845,7 +1862,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B18" t="str">
         <v>dia</v>
@@ -1871,7 +1888,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B19" t="str">
         <v>dia</v>
@@ -1897,7 +1914,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B20" t="str">
         <v>dia</v>
@@ -1923,7 +1940,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B21" t="str">
         <v>dia</v>
@@ -1949,7 +1966,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B22" t="str">
         <v>dia</v>
@@ -1975,7 +1992,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B23" t="str">
         <v>dia</v>
@@ -2001,7 +2018,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B24" t="str">
         <v>dia</v>
@@ -2027,7 +2044,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B25" t="str">
         <v>dia</v>
@@ -2053,7 +2070,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B26" t="str">
         <v>dia</v>
@@ -2079,7 +2096,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B27" t="str">
         <v>dia</v>
@@ -2105,7 +2122,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B28" t="str">
         <v>dia</v>
@@ -2131,7 +2148,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B29" t="str">
         <v>dia</v>
@@ -2157,7 +2174,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B30" t="str">
         <v>dia</v>
@@ -2183,7 +2200,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B31" t="str">
         <v>dia</v>
@@ -2209,7 +2226,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B32" t="str">
         <v>dia</v>
@@ -2235,7 +2252,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B33" t="str">
         <v>dia</v>
@@ -2261,7 +2278,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B34" t="str">
         <v>dia</v>
@@ -2287,7 +2304,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B35" t="str">
         <v>dia</v>
@@ -2313,7 +2330,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B36" t="str">
         <v>dia</v>
@@ -2337,9 +2354,35 @@
         <v/>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>2026-05</v>
+      </c>
+      <c r="B37" t="str">
+        <v>dia</v>
+      </c>
+      <c r="C37">
+        <v>31</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2539,7 +2582,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2560,13 +2603,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B2" t="str">
         <v>semana</v>
       </c>
       <c r="C2">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -2577,13 +2620,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B3" t="str">
         <v>semana</v>
       </c>
       <c r="C3">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -2594,13 +2637,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B4" t="str">
         <v>semana</v>
       </c>
       <c r="C4">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -2611,13 +2654,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B5" t="str">
         <v>semana</v>
       </c>
       <c r="C5">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -2628,13 +2671,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B6" t="str">
         <v>semana</v>
       </c>
       <c r="C6">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -2645,7 +2688,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B7" t="str">
         <v>dia</v>
@@ -2662,7 +2705,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B8" t="str">
         <v>dia</v>
@@ -2679,7 +2722,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B9" t="str">
         <v>dia</v>
@@ -2696,7 +2739,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B10" t="str">
         <v>dia</v>
@@ -2713,7 +2756,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B11" t="str">
         <v>dia</v>
@@ -2730,7 +2773,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B12" t="str">
         <v>dia</v>
@@ -2747,7 +2790,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B13" t="str">
         <v>dia</v>
@@ -2764,7 +2807,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B14" t="str">
         <v>dia</v>
@@ -2781,7 +2824,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B15" t="str">
         <v>dia</v>
@@ -2798,7 +2841,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B16" t="str">
         <v>dia</v>
@@ -2815,7 +2858,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B17" t="str">
         <v>dia</v>
@@ -2832,7 +2875,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B18" t="str">
         <v>dia</v>
@@ -2849,7 +2892,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B19" t="str">
         <v>dia</v>
@@ -2866,7 +2909,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B20" t="str">
         <v>dia</v>
@@ -2883,7 +2926,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B21" t="str">
         <v>dia</v>
@@ -2900,7 +2943,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B22" t="str">
         <v>dia</v>
@@ -2917,7 +2960,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B23" t="str">
         <v>dia</v>
@@ -2934,7 +2977,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B24" t="str">
         <v>dia</v>
@@ -2951,7 +2994,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B25" t="str">
         <v>dia</v>
@@ -2968,7 +3011,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B26" t="str">
         <v>dia</v>
@@ -2985,7 +3028,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B27" t="str">
         <v>dia</v>
@@ -3002,7 +3045,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B28" t="str">
         <v>dia</v>
@@ -3019,7 +3062,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B29" t="str">
         <v>dia</v>
@@ -3036,7 +3079,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B30" t="str">
         <v>dia</v>
@@ -3053,7 +3096,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B31" t="str">
         <v>dia</v>
@@ -3070,7 +3113,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B32" t="str">
         <v>dia</v>
@@ -3087,7 +3130,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B33" t="str">
         <v>dia</v>
@@ -3104,7 +3147,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B34" t="str">
         <v>dia</v>
@@ -3121,7 +3164,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B35" t="str">
         <v>dia</v>
@@ -3138,7 +3181,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B36" t="str">
         <v>dia</v>
@@ -3153,9 +3196,26 @@
         <v/>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>2026-05</v>
+      </c>
+      <c r="B37" t="str">
+        <v>dia</v>
+      </c>
+      <c r="C37">
+        <v>31</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3355,7 +3415,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3376,13 +3436,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B2" t="str">
         <v>semana</v>
       </c>
       <c r="C2">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -3393,13 +3453,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B3" t="str">
         <v>semana</v>
       </c>
       <c r="C3">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -3410,13 +3470,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B4" t="str">
         <v>semana</v>
       </c>
       <c r="C4">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -3427,13 +3487,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B5" t="str">
         <v>semana</v>
       </c>
       <c r="C5">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -3444,13 +3504,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B6" t="str">
         <v>semana</v>
       </c>
       <c r="C6">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -3461,7 +3521,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B7" t="str">
         <v>dia</v>
@@ -3478,7 +3538,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B8" t="str">
         <v>dia</v>
@@ -3495,7 +3555,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B9" t="str">
         <v>dia</v>
@@ -3512,7 +3572,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B10" t="str">
         <v>dia</v>
@@ -3529,7 +3589,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B11" t="str">
         <v>dia</v>
@@ -3546,7 +3606,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B12" t="str">
         <v>dia</v>
@@ -3563,7 +3623,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B13" t="str">
         <v>dia</v>
@@ -3580,7 +3640,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B14" t="str">
         <v>dia</v>
@@ -3597,7 +3657,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B15" t="str">
         <v>dia</v>
@@ -3614,7 +3674,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B16" t="str">
         <v>dia</v>
@@ -3631,7 +3691,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B17" t="str">
         <v>dia</v>
@@ -3648,7 +3708,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B18" t="str">
         <v>dia</v>
@@ -3665,7 +3725,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B19" t="str">
         <v>dia</v>
@@ -3682,7 +3742,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B20" t="str">
         <v>dia</v>
@@ -3699,7 +3759,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B21" t="str">
         <v>dia</v>
@@ -3716,7 +3776,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B22" t="str">
         <v>dia</v>
@@ -3733,7 +3793,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B23" t="str">
         <v>dia</v>
@@ -3750,7 +3810,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B24" t="str">
         <v>dia</v>
@@ -3767,7 +3827,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B25" t="str">
         <v>dia</v>
@@ -3784,7 +3844,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B26" t="str">
         <v>dia</v>
@@ -3801,7 +3861,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B27" t="str">
         <v>dia</v>
@@ -3818,7 +3878,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B28" t="str">
         <v>dia</v>
@@ -3835,7 +3895,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B29" t="str">
         <v>dia</v>
@@ -3852,7 +3912,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B30" t="str">
         <v>dia</v>
@@ -3869,7 +3929,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B31" t="str">
         <v>dia</v>
@@ -3886,7 +3946,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B32" t="str">
         <v>dia</v>
@@ -3903,7 +3963,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B33" t="str">
         <v>dia</v>
@@ -3920,7 +3980,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B34" t="str">
         <v>dia</v>
@@ -3937,7 +3997,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B35" t="str">
         <v>dia</v>
@@ -3954,7 +4014,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B36" t="str">
         <v>dia</v>
@@ -3969,9 +4029,26 @@
         <v/>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>2026-05</v>
+      </c>
+      <c r="B37" t="str">
+        <v>dia</v>
+      </c>
+      <c r="C37">
+        <v>31</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualizar plantilla de importación
</commit_message>
<xml_diff>
--- a/assets/plantilla-importacion-indicadores.xlsx
+++ b/assets/plantilla-importacion-indicadores.xlsx
@@ -430,7 +430,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2. Esta plantilla se genera con el mes de referencia: año 2026, mes 4 (2026-04).</v>
+        <v>2. Esta plantilla se genera con el mes de referencia: año 2026, mes 5 (2026-05).</v>
       </c>
     </row>
     <row r="6">
@@ -445,7 +445,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>4. En *_detalle: filas semana = semanas ISO 1-53 (como en pantalla Captura); luego filas dia = días 1-30 del mes.</v>
+        <v>4. En *_detalle: filas semana = semanas ISO 1-53 (como en pantalla Captura); luego filas dia = días 1-31 del mes.</v>
       </c>
     </row>
     <row r="9">
@@ -480,7 +480,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>carros_detalle — Semanas ISO 1-53 + un día por fila del mes (1-30), clave_mes 2026-04</v>
+        <v>carros_detalle — Semanas ISO 1-53 + un día por fila del mes (1-31), clave_mes 2026-05</v>
       </c>
     </row>
     <row r="16">
@@ -507,7 +507,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E85"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -528,7 +528,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B2" t="str">
         <v>semana</v>
@@ -545,7 +545,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B3" t="str">
         <v>semana</v>
@@ -562,7 +562,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B4" t="str">
         <v>semana</v>
@@ -579,7 +579,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B5" t="str">
         <v>semana</v>
@@ -596,7 +596,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B6" t="str">
         <v>semana</v>
@@ -613,7 +613,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B7" t="str">
         <v>semana</v>
@@ -630,7 +630,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B8" t="str">
         <v>semana</v>
@@ -647,7 +647,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B9" t="str">
         <v>semana</v>
@@ -664,7 +664,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B10" t="str">
         <v>semana</v>
@@ -681,7 +681,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B11" t="str">
         <v>semana</v>
@@ -698,7 +698,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B12" t="str">
         <v>semana</v>
@@ -715,7 +715,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B13" t="str">
         <v>semana</v>
@@ -732,7 +732,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B14" t="str">
         <v>semana</v>
@@ -749,7 +749,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B15" t="str">
         <v>semana</v>
@@ -766,7 +766,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B16" t="str">
         <v>semana</v>
@@ -783,7 +783,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B17" t="str">
         <v>semana</v>
@@ -800,7 +800,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B18" t="str">
         <v>semana</v>
@@ -817,7 +817,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B19" t="str">
         <v>semana</v>
@@ -834,7 +834,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B20" t="str">
         <v>semana</v>
@@ -851,7 +851,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B21" t="str">
         <v>semana</v>
@@ -868,7 +868,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B22" t="str">
         <v>semana</v>
@@ -885,7 +885,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B23" t="str">
         <v>semana</v>
@@ -902,7 +902,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B24" t="str">
         <v>semana</v>
@@ -919,7 +919,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B25" t="str">
         <v>semana</v>
@@ -936,7 +936,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B26" t="str">
         <v>semana</v>
@@ -953,7 +953,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B27" t="str">
         <v>semana</v>
@@ -970,7 +970,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B28" t="str">
         <v>semana</v>
@@ -987,7 +987,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B29" t="str">
         <v>semana</v>
@@ -1004,7 +1004,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B30" t="str">
         <v>semana</v>
@@ -1021,7 +1021,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B31" t="str">
         <v>semana</v>
@@ -1038,7 +1038,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B32" t="str">
         <v>semana</v>
@@ -1055,7 +1055,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B33" t="str">
         <v>semana</v>
@@ -1072,7 +1072,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B34" t="str">
         <v>semana</v>
@@ -1089,7 +1089,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B35" t="str">
         <v>semana</v>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B36" t="str">
         <v>semana</v>
@@ -1123,7 +1123,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B37" t="str">
         <v>semana</v>
@@ -1140,7 +1140,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B38" t="str">
         <v>semana</v>
@@ -1157,7 +1157,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B39" t="str">
         <v>semana</v>
@@ -1174,7 +1174,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B40" t="str">
         <v>semana</v>
@@ -1191,7 +1191,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B41" t="str">
         <v>semana</v>
@@ -1208,7 +1208,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B42" t="str">
         <v>semana</v>
@@ -1225,7 +1225,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B43" t="str">
         <v>semana</v>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B44" t="str">
         <v>semana</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B45" t="str">
         <v>semana</v>
@@ -1276,7 +1276,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B46" t="str">
         <v>semana</v>
@@ -1293,7 +1293,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B47" t="str">
         <v>semana</v>
@@ -1310,7 +1310,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B48" t="str">
         <v>semana</v>
@@ -1327,7 +1327,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B49" t="str">
         <v>semana</v>
@@ -1344,7 +1344,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B50" t="str">
         <v>semana</v>
@@ -1361,7 +1361,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B51" t="str">
         <v>semana</v>
@@ -1378,7 +1378,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B52" t="str">
         <v>semana</v>
@@ -1395,7 +1395,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B53" t="str">
         <v>semana</v>
@@ -1412,7 +1412,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B54" t="str">
         <v>semana</v>
@@ -1429,7 +1429,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B55" t="str">
         <v>dia</v>
@@ -1446,7 +1446,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B56" t="str">
         <v>dia</v>
@@ -1463,7 +1463,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B57" t="str">
         <v>dia</v>
@@ -1480,7 +1480,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B58" t="str">
         <v>dia</v>
@@ -1497,7 +1497,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B59" t="str">
         <v>dia</v>
@@ -1514,7 +1514,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B60" t="str">
         <v>dia</v>
@@ -1531,7 +1531,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B61" t="str">
         <v>dia</v>
@@ -1548,7 +1548,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B62" t="str">
         <v>dia</v>
@@ -1565,7 +1565,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B63" t="str">
         <v>dia</v>
@@ -1582,7 +1582,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B64" t="str">
         <v>dia</v>
@@ -1599,7 +1599,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B65" t="str">
         <v>dia</v>
@@ -1616,7 +1616,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B66" t="str">
         <v>dia</v>
@@ -1633,7 +1633,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B67" t="str">
         <v>dia</v>
@@ -1650,7 +1650,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B68" t="str">
         <v>dia</v>
@@ -1667,7 +1667,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B69" t="str">
         <v>dia</v>
@@ -1684,7 +1684,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B70" t="str">
         <v>dia</v>
@@ -1701,7 +1701,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B71" t="str">
         <v>dia</v>
@@ -1718,7 +1718,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B72" t="str">
         <v>dia</v>
@@ -1735,7 +1735,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B73" t="str">
         <v>dia</v>
@@ -1752,7 +1752,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B74" t="str">
         <v>dia</v>
@@ -1769,7 +1769,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B75" t="str">
         <v>dia</v>
@@ -1786,7 +1786,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B76" t="str">
         <v>dia</v>
@@ -1803,7 +1803,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B77" t="str">
         <v>dia</v>
@@ -1820,7 +1820,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B78" t="str">
         <v>dia</v>
@@ -1837,7 +1837,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B79" t="str">
         <v>dia</v>
@@ -1854,7 +1854,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B80" t="str">
         <v>dia</v>
@@ -1871,7 +1871,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B81" t="str">
         <v>dia</v>
@@ -1888,7 +1888,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B82" t="str">
         <v>dia</v>
@@ -1905,7 +1905,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B83" t="str">
         <v>dia</v>
@@ -1922,7 +1922,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B84" t="str">
         <v>dia</v>
@@ -1937,9 +1937,26 @@
         <v/>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>2026-05</v>
+      </c>
+      <c r="B85" t="str">
+        <v>dia</v>
+      </c>
+      <c r="C85">
+        <v>31</v>
+      </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E84"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E85"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2215,7 +2232,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H85"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2245,7 +2262,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B2" t="str">
         <v>semana</v>
@@ -2271,7 +2288,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B3" t="str">
         <v>semana</v>
@@ -2297,7 +2314,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B4" t="str">
         <v>semana</v>
@@ -2323,7 +2340,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B5" t="str">
         <v>semana</v>
@@ -2349,7 +2366,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B6" t="str">
         <v>semana</v>
@@ -2375,7 +2392,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B7" t="str">
         <v>semana</v>
@@ -2401,7 +2418,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B8" t="str">
         <v>semana</v>
@@ -2427,7 +2444,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B9" t="str">
         <v>semana</v>
@@ -2453,7 +2470,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B10" t="str">
         <v>semana</v>
@@ -2479,7 +2496,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B11" t="str">
         <v>semana</v>
@@ -2505,7 +2522,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B12" t="str">
         <v>semana</v>
@@ -2531,7 +2548,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B13" t="str">
         <v>semana</v>
@@ -2557,7 +2574,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B14" t="str">
         <v>semana</v>
@@ -2583,7 +2600,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B15" t="str">
         <v>semana</v>
@@ -2609,7 +2626,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B16" t="str">
         <v>semana</v>
@@ -2635,7 +2652,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B17" t="str">
         <v>semana</v>
@@ -2661,7 +2678,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B18" t="str">
         <v>semana</v>
@@ -2687,7 +2704,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B19" t="str">
         <v>semana</v>
@@ -2713,7 +2730,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B20" t="str">
         <v>semana</v>
@@ -2739,7 +2756,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B21" t="str">
         <v>semana</v>
@@ -2765,7 +2782,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B22" t="str">
         <v>semana</v>
@@ -2791,7 +2808,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B23" t="str">
         <v>semana</v>
@@ -2817,7 +2834,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B24" t="str">
         <v>semana</v>
@@ -2843,7 +2860,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B25" t="str">
         <v>semana</v>
@@ -2869,7 +2886,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B26" t="str">
         <v>semana</v>
@@ -2895,7 +2912,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B27" t="str">
         <v>semana</v>
@@ -2921,7 +2938,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B28" t="str">
         <v>semana</v>
@@ -2947,7 +2964,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B29" t="str">
         <v>semana</v>
@@ -2973,7 +2990,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B30" t="str">
         <v>semana</v>
@@ -2999,7 +3016,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B31" t="str">
         <v>semana</v>
@@ -3025,7 +3042,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B32" t="str">
         <v>semana</v>
@@ -3051,7 +3068,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B33" t="str">
         <v>semana</v>
@@ -3077,7 +3094,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B34" t="str">
         <v>semana</v>
@@ -3103,7 +3120,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B35" t="str">
         <v>semana</v>
@@ -3129,7 +3146,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B36" t="str">
         <v>semana</v>
@@ -3155,7 +3172,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B37" t="str">
         <v>semana</v>
@@ -3181,7 +3198,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B38" t="str">
         <v>semana</v>
@@ -3207,7 +3224,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B39" t="str">
         <v>semana</v>
@@ -3233,7 +3250,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B40" t="str">
         <v>semana</v>
@@ -3259,7 +3276,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B41" t="str">
         <v>semana</v>
@@ -3285,7 +3302,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B42" t="str">
         <v>semana</v>
@@ -3311,7 +3328,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B43" t="str">
         <v>semana</v>
@@ -3337,7 +3354,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B44" t="str">
         <v>semana</v>
@@ -3363,7 +3380,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B45" t="str">
         <v>semana</v>
@@ -3389,7 +3406,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B46" t="str">
         <v>semana</v>
@@ -3415,7 +3432,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B47" t="str">
         <v>semana</v>
@@ -3441,7 +3458,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B48" t="str">
         <v>semana</v>
@@ -3467,7 +3484,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B49" t="str">
         <v>semana</v>
@@ -3493,7 +3510,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B50" t="str">
         <v>semana</v>
@@ -3519,7 +3536,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B51" t="str">
         <v>semana</v>
@@ -3545,7 +3562,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B52" t="str">
         <v>semana</v>
@@ -3571,7 +3588,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B53" t="str">
         <v>semana</v>
@@ -3597,7 +3614,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B54" t="str">
         <v>semana</v>
@@ -3623,7 +3640,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B55" t="str">
         <v>dia</v>
@@ -3649,7 +3666,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B56" t="str">
         <v>dia</v>
@@ -3675,7 +3692,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B57" t="str">
         <v>dia</v>
@@ -3701,7 +3718,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B58" t="str">
         <v>dia</v>
@@ -3727,7 +3744,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B59" t="str">
         <v>dia</v>
@@ -3753,7 +3770,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B60" t="str">
         <v>dia</v>
@@ -3779,7 +3796,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B61" t="str">
         <v>dia</v>
@@ -3805,7 +3822,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B62" t="str">
         <v>dia</v>
@@ -3831,7 +3848,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B63" t="str">
         <v>dia</v>
@@ -3857,7 +3874,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B64" t="str">
         <v>dia</v>
@@ -3883,7 +3900,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B65" t="str">
         <v>dia</v>
@@ -3909,7 +3926,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B66" t="str">
         <v>dia</v>
@@ -3935,7 +3952,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B67" t="str">
         <v>dia</v>
@@ -3961,7 +3978,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B68" t="str">
         <v>dia</v>
@@ -3987,7 +4004,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B69" t="str">
         <v>dia</v>
@@ -4013,7 +4030,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B70" t="str">
         <v>dia</v>
@@ -4039,7 +4056,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B71" t="str">
         <v>dia</v>
@@ -4065,7 +4082,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B72" t="str">
         <v>dia</v>
@@ -4091,7 +4108,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B73" t="str">
         <v>dia</v>
@@ -4117,7 +4134,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B74" t="str">
         <v>dia</v>
@@ -4143,7 +4160,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B75" t="str">
         <v>dia</v>
@@ -4169,7 +4186,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B76" t="str">
         <v>dia</v>
@@ -4195,7 +4212,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B77" t="str">
         <v>dia</v>
@@ -4221,7 +4238,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B78" t="str">
         <v>dia</v>
@@ -4247,7 +4264,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B79" t="str">
         <v>dia</v>
@@ -4273,7 +4290,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B80" t="str">
         <v>dia</v>
@@ -4299,7 +4316,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B81" t="str">
         <v>dia</v>
@@ -4325,7 +4342,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B82" t="str">
         <v>dia</v>
@@ -4351,7 +4368,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B83" t="str">
         <v>dia</v>
@@ -4377,7 +4394,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B84" t="str">
         <v>dia</v>
@@ -4401,9 +4418,35 @@
         <v/>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>2026-05</v>
+      </c>
+      <c r="B85" t="str">
+        <v>dia</v>
+      </c>
+      <c r="C85">
+        <v>31</v>
+      </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
+      <c r="F85" t="str">
+        <v/>
+      </c>
+      <c r="G85" t="str">
+        <v/>
+      </c>
+      <c r="H85" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H84"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H85"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4603,7 +4646,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E85"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4624,7 +4667,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B2" t="str">
         <v>semana</v>
@@ -4641,7 +4684,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B3" t="str">
         <v>semana</v>
@@ -4658,7 +4701,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B4" t="str">
         <v>semana</v>
@@ -4675,7 +4718,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B5" t="str">
         <v>semana</v>
@@ -4692,7 +4735,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B6" t="str">
         <v>semana</v>
@@ -4709,7 +4752,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B7" t="str">
         <v>semana</v>
@@ -4726,7 +4769,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B8" t="str">
         <v>semana</v>
@@ -4743,7 +4786,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B9" t="str">
         <v>semana</v>
@@ -4760,7 +4803,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B10" t="str">
         <v>semana</v>
@@ -4777,7 +4820,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B11" t="str">
         <v>semana</v>
@@ -4794,7 +4837,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B12" t="str">
         <v>semana</v>
@@ -4811,7 +4854,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B13" t="str">
         <v>semana</v>
@@ -4828,7 +4871,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B14" t="str">
         <v>semana</v>
@@ -4845,7 +4888,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B15" t="str">
         <v>semana</v>
@@ -4862,7 +4905,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B16" t="str">
         <v>semana</v>
@@ -4879,7 +4922,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B17" t="str">
         <v>semana</v>
@@ -4896,7 +4939,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B18" t="str">
         <v>semana</v>
@@ -4913,7 +4956,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B19" t="str">
         <v>semana</v>
@@ -4930,7 +4973,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B20" t="str">
         <v>semana</v>
@@ -4947,7 +4990,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B21" t="str">
         <v>semana</v>
@@ -4964,7 +5007,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B22" t="str">
         <v>semana</v>
@@ -4981,7 +5024,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B23" t="str">
         <v>semana</v>
@@ -4998,7 +5041,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B24" t="str">
         <v>semana</v>
@@ -5015,7 +5058,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B25" t="str">
         <v>semana</v>
@@ -5032,7 +5075,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B26" t="str">
         <v>semana</v>
@@ -5049,7 +5092,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B27" t="str">
         <v>semana</v>
@@ -5066,7 +5109,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B28" t="str">
         <v>semana</v>
@@ -5083,7 +5126,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B29" t="str">
         <v>semana</v>
@@ -5100,7 +5143,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B30" t="str">
         <v>semana</v>
@@ -5117,7 +5160,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B31" t="str">
         <v>semana</v>
@@ -5134,7 +5177,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B32" t="str">
         <v>semana</v>
@@ -5151,7 +5194,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B33" t="str">
         <v>semana</v>
@@ -5168,7 +5211,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B34" t="str">
         <v>semana</v>
@@ -5185,7 +5228,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B35" t="str">
         <v>semana</v>
@@ -5202,7 +5245,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B36" t="str">
         <v>semana</v>
@@ -5219,7 +5262,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B37" t="str">
         <v>semana</v>
@@ -5236,7 +5279,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B38" t="str">
         <v>semana</v>
@@ -5253,7 +5296,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B39" t="str">
         <v>semana</v>
@@ -5270,7 +5313,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B40" t="str">
         <v>semana</v>
@@ -5287,7 +5330,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B41" t="str">
         <v>semana</v>
@@ -5304,7 +5347,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B42" t="str">
         <v>semana</v>
@@ -5321,7 +5364,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B43" t="str">
         <v>semana</v>
@@ -5338,7 +5381,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B44" t="str">
         <v>semana</v>
@@ -5355,7 +5398,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B45" t="str">
         <v>semana</v>
@@ -5372,7 +5415,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B46" t="str">
         <v>semana</v>
@@ -5389,7 +5432,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B47" t="str">
         <v>semana</v>
@@ -5406,7 +5449,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B48" t="str">
         <v>semana</v>
@@ -5423,7 +5466,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B49" t="str">
         <v>semana</v>
@@ -5440,7 +5483,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B50" t="str">
         <v>semana</v>
@@ -5457,7 +5500,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B51" t="str">
         <v>semana</v>
@@ -5474,7 +5517,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B52" t="str">
         <v>semana</v>
@@ -5491,7 +5534,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B53" t="str">
         <v>semana</v>
@@ -5508,7 +5551,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B54" t="str">
         <v>semana</v>
@@ -5525,7 +5568,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B55" t="str">
         <v>dia</v>
@@ -5542,7 +5585,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B56" t="str">
         <v>dia</v>
@@ -5559,7 +5602,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B57" t="str">
         <v>dia</v>
@@ -5576,7 +5619,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B58" t="str">
         <v>dia</v>
@@ -5593,7 +5636,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B59" t="str">
         <v>dia</v>
@@ -5610,7 +5653,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B60" t="str">
         <v>dia</v>
@@ -5627,7 +5670,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B61" t="str">
         <v>dia</v>
@@ -5644,7 +5687,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B62" t="str">
         <v>dia</v>
@@ -5661,7 +5704,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B63" t="str">
         <v>dia</v>
@@ -5678,7 +5721,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B64" t="str">
         <v>dia</v>
@@ -5695,7 +5738,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B65" t="str">
         <v>dia</v>
@@ -5712,7 +5755,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B66" t="str">
         <v>dia</v>
@@ -5729,7 +5772,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B67" t="str">
         <v>dia</v>
@@ -5746,7 +5789,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B68" t="str">
         <v>dia</v>
@@ -5763,7 +5806,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B69" t="str">
         <v>dia</v>
@@ -5780,7 +5823,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B70" t="str">
         <v>dia</v>
@@ -5797,7 +5840,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B71" t="str">
         <v>dia</v>
@@ -5814,7 +5857,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B72" t="str">
         <v>dia</v>
@@ -5831,7 +5874,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B73" t="str">
         <v>dia</v>
@@ -5848,7 +5891,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B74" t="str">
         <v>dia</v>
@@ -5865,7 +5908,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B75" t="str">
         <v>dia</v>
@@ -5882,7 +5925,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B76" t="str">
         <v>dia</v>
@@ -5899,7 +5942,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B77" t="str">
         <v>dia</v>
@@ -5916,7 +5959,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B78" t="str">
         <v>dia</v>
@@ -5933,7 +5976,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B79" t="str">
         <v>dia</v>
@@ -5950,7 +5993,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B80" t="str">
         <v>dia</v>
@@ -5967,7 +6010,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B81" t="str">
         <v>dia</v>
@@ -5984,7 +6027,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B82" t="str">
         <v>dia</v>
@@ -6001,7 +6044,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B83" t="str">
         <v>dia</v>
@@ -6018,7 +6061,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B84" t="str">
         <v>dia</v>
@@ -6033,9 +6076,26 @@
         <v/>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>2026-05</v>
+      </c>
+      <c r="B85" t="str">
+        <v>dia</v>
+      </c>
+      <c r="C85">
+        <v>31</v>
+      </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E84"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E85"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6235,7 +6295,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E85"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6256,7 +6316,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B2" t="str">
         <v>semana</v>
@@ -6273,7 +6333,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B3" t="str">
         <v>semana</v>
@@ -6290,7 +6350,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B4" t="str">
         <v>semana</v>
@@ -6307,7 +6367,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B5" t="str">
         <v>semana</v>
@@ -6324,7 +6384,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B6" t="str">
         <v>semana</v>
@@ -6341,7 +6401,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B7" t="str">
         <v>semana</v>
@@ -6358,7 +6418,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B8" t="str">
         <v>semana</v>
@@ -6375,7 +6435,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B9" t="str">
         <v>semana</v>
@@ -6392,7 +6452,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B10" t="str">
         <v>semana</v>
@@ -6409,7 +6469,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B11" t="str">
         <v>semana</v>
@@ -6426,7 +6486,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B12" t="str">
         <v>semana</v>
@@ -6443,7 +6503,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B13" t="str">
         <v>semana</v>
@@ -6460,7 +6520,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B14" t="str">
         <v>semana</v>
@@ -6477,7 +6537,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B15" t="str">
         <v>semana</v>
@@ -6494,7 +6554,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B16" t="str">
         <v>semana</v>
@@ -6511,7 +6571,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B17" t="str">
         <v>semana</v>
@@ -6528,7 +6588,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B18" t="str">
         <v>semana</v>
@@ -6545,7 +6605,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B19" t="str">
         <v>semana</v>
@@ -6562,7 +6622,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B20" t="str">
         <v>semana</v>
@@ -6579,7 +6639,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B21" t="str">
         <v>semana</v>
@@ -6596,7 +6656,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B22" t="str">
         <v>semana</v>
@@ -6613,7 +6673,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B23" t="str">
         <v>semana</v>
@@ -6630,7 +6690,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B24" t="str">
         <v>semana</v>
@@ -6647,7 +6707,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B25" t="str">
         <v>semana</v>
@@ -6664,7 +6724,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B26" t="str">
         <v>semana</v>
@@ -6681,7 +6741,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B27" t="str">
         <v>semana</v>
@@ -6698,7 +6758,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B28" t="str">
         <v>semana</v>
@@ -6715,7 +6775,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B29" t="str">
         <v>semana</v>
@@ -6732,7 +6792,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B30" t="str">
         <v>semana</v>
@@ -6749,7 +6809,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B31" t="str">
         <v>semana</v>
@@ -6766,7 +6826,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B32" t="str">
         <v>semana</v>
@@ -6783,7 +6843,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B33" t="str">
         <v>semana</v>
@@ -6800,7 +6860,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B34" t="str">
         <v>semana</v>
@@ -6817,7 +6877,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B35" t="str">
         <v>semana</v>
@@ -6834,7 +6894,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B36" t="str">
         <v>semana</v>
@@ -6851,7 +6911,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B37" t="str">
         <v>semana</v>
@@ -6868,7 +6928,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B38" t="str">
         <v>semana</v>
@@ -6885,7 +6945,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B39" t="str">
         <v>semana</v>
@@ -6902,7 +6962,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B40" t="str">
         <v>semana</v>
@@ -6919,7 +6979,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B41" t="str">
         <v>semana</v>
@@ -6936,7 +6996,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B42" t="str">
         <v>semana</v>
@@ -6953,7 +7013,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B43" t="str">
         <v>semana</v>
@@ -6970,7 +7030,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B44" t="str">
         <v>semana</v>
@@ -6987,7 +7047,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B45" t="str">
         <v>semana</v>
@@ -7004,7 +7064,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B46" t="str">
         <v>semana</v>
@@ -7021,7 +7081,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B47" t="str">
         <v>semana</v>
@@ -7038,7 +7098,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B48" t="str">
         <v>semana</v>
@@ -7055,7 +7115,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B49" t="str">
         <v>semana</v>
@@ -7072,7 +7132,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B50" t="str">
         <v>semana</v>
@@ -7089,7 +7149,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B51" t="str">
         <v>semana</v>
@@ -7106,7 +7166,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B52" t="str">
         <v>semana</v>
@@ -7123,7 +7183,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B53" t="str">
         <v>semana</v>
@@ -7140,7 +7200,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B54" t="str">
         <v>semana</v>
@@ -7157,7 +7217,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B55" t="str">
         <v>dia</v>
@@ -7174,7 +7234,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B56" t="str">
         <v>dia</v>
@@ -7191,7 +7251,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B57" t="str">
         <v>dia</v>
@@ -7208,7 +7268,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B58" t="str">
         <v>dia</v>
@@ -7225,7 +7285,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B59" t="str">
         <v>dia</v>
@@ -7242,7 +7302,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B60" t="str">
         <v>dia</v>
@@ -7259,7 +7319,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B61" t="str">
         <v>dia</v>
@@ -7276,7 +7336,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B62" t="str">
         <v>dia</v>
@@ -7293,7 +7353,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B63" t="str">
         <v>dia</v>
@@ -7310,7 +7370,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B64" t="str">
         <v>dia</v>
@@ -7327,7 +7387,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B65" t="str">
         <v>dia</v>
@@ -7344,7 +7404,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B66" t="str">
         <v>dia</v>
@@ -7361,7 +7421,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B67" t="str">
         <v>dia</v>
@@ -7378,7 +7438,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B68" t="str">
         <v>dia</v>
@@ -7395,7 +7455,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B69" t="str">
         <v>dia</v>
@@ -7412,7 +7472,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B70" t="str">
         <v>dia</v>
@@ -7429,7 +7489,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B71" t="str">
         <v>dia</v>
@@ -7446,7 +7506,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B72" t="str">
         <v>dia</v>
@@ -7463,7 +7523,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B73" t="str">
         <v>dia</v>
@@ -7480,7 +7540,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B74" t="str">
         <v>dia</v>
@@ -7497,7 +7557,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B75" t="str">
         <v>dia</v>
@@ -7514,7 +7574,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B76" t="str">
         <v>dia</v>
@@ -7531,7 +7591,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B77" t="str">
         <v>dia</v>
@@ -7548,7 +7608,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B78" t="str">
         <v>dia</v>
@@ -7565,7 +7625,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B79" t="str">
         <v>dia</v>
@@ -7582,7 +7642,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B80" t="str">
         <v>dia</v>
@@ -7599,7 +7659,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B81" t="str">
         <v>dia</v>
@@ -7616,7 +7676,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B82" t="str">
         <v>dia</v>
@@ -7633,7 +7693,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B83" t="str">
         <v>dia</v>
@@ -7650,7 +7710,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2026-04</v>
+        <v>2026-05</v>
       </c>
       <c r="B84" t="str">
         <v>dia</v>
@@ -7665,9 +7725,26 @@
         <v/>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>2026-05</v>
+      </c>
+      <c r="B85" t="str">
+        <v>dia</v>
+      </c>
+      <c r="C85">
+        <v>31</v>
+      </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E84"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E85"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>